<commit_message>
Updated DEU_grids_kan model - 2025-12-05 16:37
</commit_message>
<xml_diff>
--- a/VerveStacks_DEU_grids_kan/Sets-vervestacks.xlsx
+++ b/VerveStacks_DEU_grids_kan/Sets-vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_DEU_grids_kan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3A5A8A66-E87F-49D3-8551-818B0D1DCBB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{CBED39E9-C5BA-4E1C-AC83-230EF8D8053B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4355,7 +4355,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{57D96054-D1EA-4044-B06F-7638DAEDECA0}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{458BB755-7186-461E-B6C1-F2EF2DC81E7E}">
   <dimension ref="B9:E538"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>

</xml_diff>